<commit_message>
Continued adjustments and error searching
</commit_message>
<xml_diff>
--- a/Processed_Data/PM25_check.xlsx
+++ b/Processed_Data/PM25_check.xlsx
@@ -13675,13 +13675,13 @@
         </is>
       </c>
       <c r="D552" t="n">
-        <v>4.3</v>
+        <v>4.237</v>
       </c>
       <c r="E552" t="n">
-        <v>39166</v>
+        <v>38546</v>
       </c>
       <c r="F552" t="n">
-        <v>3956</v>
+        <v>3893</v>
       </c>
     </row>
     <row r="553">
@@ -13699,13 +13699,13 @@
         </is>
       </c>
       <c r="D553" t="n">
-        <v>5.34</v>
+        <v>5.232</v>
       </c>
       <c r="E553" t="n">
-        <v>62442</v>
+        <v>61162</v>
       </c>
       <c r="F553" t="n">
-        <v>6204</v>
+        <v>6077</v>
       </c>
     </row>
     <row r="554">
@@ -13723,13 +13723,13 @@
         </is>
       </c>
       <c r="D554" t="n">
-        <v>5.83</v>
+        <v>5.752</v>
       </c>
       <c r="E554" t="n">
-        <v>51282</v>
+        <v>50573</v>
       </c>
       <c r="F554" t="n">
-        <v>5058</v>
+        <v>4988</v>
       </c>
     </row>
     <row r="555">
@@ -13747,13 +13747,13 @@
         </is>
       </c>
       <c r="D555" t="n">
-        <v>4.68</v>
+        <v>4.613</v>
       </c>
       <c r="E555" t="n">
-        <v>21197</v>
+        <v>20911</v>
       </c>
       <c r="F555" t="n">
-        <v>2205</v>
+        <v>2175</v>
       </c>
     </row>
     <row r="556">
@@ -13771,13 +13771,13 @@
         </is>
       </c>
       <c r="D556" t="n">
-        <v>6.03</v>
+        <v>5.975</v>
       </c>
       <c r="E556" t="n">
-        <v>7246</v>
+        <v>7180</v>
       </c>
       <c r="F556" t="n">
-        <v>667</v>
+        <v>661</v>
       </c>
     </row>
     <row r="557">
@@ -13795,13 +13795,13 @@
         </is>
       </c>
       <c r="D557" t="n">
-        <v>4.87</v>
+        <v>4.8</v>
       </c>
       <c r="E557" t="n">
-        <v>56656</v>
+        <v>55899</v>
       </c>
       <c r="F557" t="n">
-        <v>5809</v>
+        <v>5732</v>
       </c>
     </row>
     <row r="558">
@@ -13819,13 +13819,13 @@
         </is>
       </c>
       <c r="D558" t="n">
-        <v>3.47</v>
+        <v>3.405</v>
       </c>
       <c r="E558" t="n">
-        <v>20198</v>
+        <v>19839</v>
       </c>
       <c r="F558" t="n">
-        <v>2130</v>
+        <v>2092</v>
       </c>
     </row>
     <row r="559">
@@ -13843,13 +13843,13 @@
         </is>
       </c>
       <c r="D559" t="n">
-        <v>3.21</v>
+        <v>3.17</v>
       </c>
       <c r="E559" t="n">
-        <v>5165</v>
+        <v>5106</v>
       </c>
       <c r="F559" t="n">
-        <v>478</v>
+        <v>473</v>
       </c>
     </row>
     <row r="560">
@@ -13867,13 +13867,13 @@
         </is>
       </c>
       <c r="D560" t="n">
-        <v>2.48</v>
+        <v>2.443</v>
       </c>
       <c r="E560" t="n">
-        <v>14172</v>
+        <v>13990</v>
       </c>
       <c r="F560" t="n">
-        <v>1555</v>
+        <v>1535</v>
       </c>
     </row>
     <row r="561">
@@ -13891,13 +13891,13 @@
         </is>
       </c>
       <c r="D561" t="n">
-        <v>3.98</v>
+        <v>3.907</v>
       </c>
       <c r="E561" t="n">
-        <v>269312</v>
+        <v>264111</v>
       </c>
       <c r="F561" t="n">
-        <v>26517</v>
+        <v>26004</v>
       </c>
     </row>
     <row r="562">
@@ -13915,13 +13915,13 @@
         </is>
       </c>
       <c r="D562" t="n">
-        <v>4.29</v>
+        <v>4.225</v>
       </c>
       <c r="E562" t="n">
-        <v>384949</v>
+        <v>378636</v>
       </c>
       <c r="F562" t="n">
-        <v>39754</v>
+        <v>39102</v>
       </c>
     </row>
     <row r="563">
@@ -13939,13 +13939,13 @@
         </is>
       </c>
       <c r="D563" t="n">
-        <v>6.73</v>
+        <v>6.635</v>
       </c>
       <c r="E563" t="n">
-        <v>74059</v>
+        <v>72976</v>
       </c>
       <c r="F563" t="n">
-        <v>7436</v>
+        <v>7327</v>
       </c>
     </row>
     <row r="564">
@@ -13963,13 +13963,13 @@
         </is>
       </c>
       <c r="D564" t="n">
-        <v>5.76</v>
+        <v>5.688</v>
       </c>
       <c r="E564" t="n">
-        <v>72438</v>
+        <v>71526</v>
       </c>
       <c r="F564" t="n">
-        <v>6713</v>
+        <v>6628</v>
       </c>
     </row>
     <row r="565">
@@ -13987,13 +13987,13 @@
         </is>
       </c>
       <c r="D565" t="n">
-        <v>2.06</v>
+        <v>2.029</v>
       </c>
       <c r="E565" t="n">
-        <v>9422</v>
+        <v>9262</v>
       </c>
       <c r="F565" t="n">
-        <v>902</v>
+        <v>886</v>
       </c>
     </row>
     <row r="566">
@@ -14011,13 +14011,13 @@
         </is>
       </c>
       <c r="D566" t="n">
-        <v>6.88</v>
+        <v>6.773</v>
       </c>
       <c r="E566" t="n">
-        <v>400464</v>
+        <v>393907</v>
       </c>
       <c r="F566" t="n">
-        <v>44541</v>
+        <v>43812</v>
       </c>
     </row>
     <row r="567">
@@ -14035,13 +14035,13 @@
         </is>
       </c>
       <c r="D567" t="n">
-        <v>3.79</v>
+        <v>3.751</v>
       </c>
       <c r="E567" t="n">
-        <v>9657</v>
+        <v>9547</v>
       </c>
       <c r="F567" t="n">
-        <v>871</v>
+        <v>861</v>
       </c>
     </row>
     <row r="568">
@@ -14059,13 +14059,13 @@
         </is>
       </c>
       <c r="D568" t="n">
-        <v>4.01</v>
+        <v>3.964</v>
       </c>
       <c r="E568" t="n">
-        <v>15459</v>
+        <v>15283</v>
       </c>
       <c r="F568" t="n">
-        <v>1353</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="569">
@@ -14083,13 +14083,13 @@
         </is>
       </c>
       <c r="D569" t="n">
-        <v>4</v>
+        <v>3.941</v>
       </c>
       <c r="E569" t="n">
-        <v>2520</v>
+        <v>2483</v>
       </c>
       <c r="F569" t="n">
-        <v>229</v>
+        <v>225</v>
       </c>
     </row>
     <row r="570">
@@ -14107,13 +14107,13 @@
         </is>
       </c>
       <c r="D570" t="n">
-        <v>6.95</v>
+        <v>6.9</v>
       </c>
       <c r="E570" t="n">
-        <v>3856</v>
+        <v>3828</v>
       </c>
       <c r="F570" t="n">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="571">
@@ -14131,13 +14131,13 @@
         </is>
       </c>
       <c r="D571" t="n">
-        <v>5.68</v>
+        <v>5.513</v>
       </c>
       <c r="E571" t="n">
-        <v>97775</v>
+        <v>94875</v>
       </c>
       <c r="F571" t="n">
-        <v>10579</v>
+        <v>10265</v>
       </c>
     </row>
     <row r="572">
@@ -14155,13 +14155,13 @@
         </is>
       </c>
       <c r="D572" t="n">
-        <v>4.74</v>
+        <v>4.662</v>
       </c>
       <c r="E572" t="n">
-        <v>225126</v>
+        <v>221310</v>
       </c>
       <c r="F572" t="n">
-        <v>20223</v>
+        <v>19880</v>
       </c>
     </row>
     <row r="573">
@@ -14179,13 +14179,13 @@
         </is>
       </c>
       <c r="D573" t="n">
-        <v>4.3</v>
+        <v>4.256</v>
       </c>
       <c r="E573" t="n">
-        <v>48483</v>
+        <v>47947</v>
       </c>
       <c r="F573" t="n">
-        <v>5041</v>
+        <v>4985</v>
       </c>
     </row>
     <row r="574">
@@ -14203,13 +14203,13 @@
         </is>
       </c>
       <c r="D574" t="n">
-        <v>7</v>
+        <v>6.928</v>
       </c>
       <c r="E574" t="n">
-        <v>166743</v>
+        <v>165076</v>
       </c>
       <c r="F574" t="n">
-        <v>15950</v>
+        <v>15791</v>
       </c>
     </row>
     <row r="575">
@@ -14227,13 +14227,13 @@
         </is>
       </c>
       <c r="D575" t="n">
-        <v>4.71</v>
+        <v>4.644</v>
       </c>
       <c r="E575" t="n">
-        <v>30760</v>
+        <v>30348</v>
       </c>
       <c r="F575" t="n">
-        <v>2841</v>
+        <v>2803</v>
       </c>
     </row>
     <row r="576">
@@ -14251,13 +14251,13 @@
         </is>
       </c>
       <c r="D576" t="n">
-        <v>6.25</v>
+        <v>6.169</v>
       </c>
       <c r="E576" t="n">
-        <v>14600</v>
+        <v>14423</v>
       </c>
       <c r="F576" t="n">
-        <v>1435</v>
+        <v>1417</v>
       </c>
     </row>
     <row r="577">
@@ -14275,13 +14275,13 @@
         </is>
       </c>
       <c r="D577" t="n">
-        <v>4.74</v>
+        <v>4.664</v>
       </c>
       <c r="E577" t="n">
-        <v>223505</v>
+        <v>220039</v>
       </c>
       <c r="F577" t="n">
-        <v>22395</v>
+        <v>22048</v>
       </c>
     </row>
     <row r="578">
@@ -14299,13 +14299,13 @@
         </is>
       </c>
       <c r="D578" t="n">
-        <v>2.58</v>
+        <v>2.543</v>
       </c>
       <c r="E578" t="n">
-        <v>23606</v>
+        <v>23281</v>
       </c>
       <c r="F578" t="n">
-        <v>2627</v>
+        <v>2591</v>
       </c>
     </row>
     <row r="579">
@@ -14323,13 +14323,13 @@
         </is>
       </c>
       <c r="D579" t="n">
-        <v>10.52</v>
+        <v>10.397</v>
       </c>
       <c r="E579" t="n">
-        <v>27607</v>
+        <v>27297</v>
       </c>
       <c r="F579" t="n">
-        <v>2700</v>
+        <v>2670</v>
       </c>
     </row>
     <row r="580">
@@ -14347,13 +14347,13 @@
         </is>
       </c>
       <c r="D580" t="n">
-        <v>21.19</v>
+        <v>20.923</v>
       </c>
       <c r="E580" t="n">
-        <v>69285</v>
+        <v>68417</v>
       </c>
       <c r="F580" t="n">
-        <v>6170</v>
+        <v>6092</v>
       </c>
     </row>
     <row r="581">
@@ -14371,13 +14371,13 @@
         </is>
       </c>
       <c r="D581" t="n">
-        <v>11.82</v>
+        <v>11.64</v>
       </c>
       <c r="E581" t="n">
-        <v>130147</v>
+        <v>128126</v>
       </c>
       <c r="F581" t="n">
-        <v>10768</v>
+        <v>10601</v>
       </c>
     </row>
     <row r="582">
@@ -14395,13 +14395,13 @@
         </is>
       </c>
       <c r="D582" t="n">
-        <v>6.75</v>
+        <v>6.639</v>
       </c>
       <c r="E582" t="n">
-        <v>85021</v>
+        <v>83683</v>
       </c>
       <c r="F582" t="n">
-        <v>7428</v>
+        <v>7311</v>
       </c>
     </row>
     <row r="583">
@@ -14419,13 +14419,13 @@
         </is>
       </c>
       <c r="D583" t="n">
-        <v>12.18</v>
+        <v>12.068</v>
       </c>
       <c r="E583" t="n">
-        <v>49836</v>
+        <v>49377</v>
       </c>
       <c r="F583" t="n">
-        <v>4751</v>
+        <v>4707</v>
       </c>
     </row>
     <row r="584">
@@ -14443,13 +14443,13 @@
         </is>
       </c>
       <c r="D584" t="n">
-        <v>11.03</v>
+        <v>10.866</v>
       </c>
       <c r="E584" t="n">
-        <v>52917</v>
+        <v>52143</v>
       </c>
       <c r="F584" t="n">
-        <v>4537</v>
+        <v>4471</v>
       </c>
     </row>
     <row r="585">
@@ -14467,10 +14467,10 @@
         </is>
       </c>
       <c r="D585" t="n">
-        <v>3.12</v>
+        <v>3.114</v>
       </c>
       <c r="E585" t="n">
-        <v>966</v>
+        <v>965</v>
       </c>
       <c r="F585" t="n">
         <v>99</v>
@@ -14491,13 +14491,13 @@
         </is>
       </c>
       <c r="D586" t="n">
-        <v>20.63</v>
+        <v>20.099</v>
       </c>
       <c r="E586" t="n">
-        <v>466739</v>
+        <v>454722</v>
       </c>
       <c r="F586" t="n">
-        <v>34308</v>
+        <v>33425</v>
       </c>
     </row>
     <row r="587">
@@ -14515,13 +14515,13 @@
         </is>
       </c>
       <c r="D587" t="n">
-        <v>18.06</v>
+        <v>17.957</v>
       </c>
       <c r="E587" t="n">
-        <v>24849</v>
+        <v>24709</v>
       </c>
       <c r="F587" t="n">
-        <v>2191</v>
+        <v>2179</v>
       </c>
     </row>
     <row r="588">
@@ -14539,13 +14539,13 @@
         </is>
       </c>
       <c r="D588" t="n">
-        <v>14.86</v>
+        <v>14.522</v>
       </c>
       <c r="E588" t="n">
-        <v>106939</v>
+        <v>104536</v>
       </c>
       <c r="F588" t="n">
-        <v>7972</v>
+        <v>7793</v>
       </c>
     </row>
     <row r="589">
@@ -14563,13 +14563,13 @@
         </is>
       </c>
       <c r="D589" t="n">
-        <v>9.470000000000001</v>
+        <v>9.372999999999999</v>
       </c>
       <c r="E589" t="n">
-        <v>19076</v>
+        <v>18884</v>
       </c>
       <c r="F589" t="n">
-        <v>1941</v>
+        <v>1921</v>
       </c>
     </row>
     <row r="590">
@@ -14587,13 +14587,13 @@
         </is>
       </c>
       <c r="D590" t="n">
-        <v>9.27</v>
+        <v>9.163</v>
       </c>
       <c r="E590" t="n">
-        <v>39481</v>
+        <v>39040</v>
       </c>
       <c r="F590" t="n">
-        <v>3480</v>
+        <v>3441</v>
       </c>
     </row>
     <row r="591">
@@ -14611,13 +14611,13 @@
         </is>
       </c>
       <c r="D591" t="n">
-        <v>13.02</v>
+        <v>12.969</v>
       </c>
       <c r="E591" t="n">
-        <v>9377</v>
+        <v>9338</v>
       </c>
       <c r="F591" t="n">
-        <v>878</v>
+        <v>874</v>
       </c>
     </row>
     <row r="592">
@@ -14635,13 +14635,13 @@
         </is>
       </c>
       <c r="D592" t="n">
-        <v>2.41</v>
+        <v>2.386</v>
       </c>
       <c r="E592" t="n">
-        <v>11665</v>
+        <v>11542</v>
       </c>
       <c r="F592" t="n">
-        <v>1231</v>
+        <v>1218</v>
       </c>
     </row>
     <row r="593">
@@ -14659,13 +14659,13 @@
         </is>
       </c>
       <c r="D593" t="n">
-        <v>9.25</v>
+        <v>8.961</v>
       </c>
       <c r="E593" t="n">
-        <v>1525673</v>
+        <v>1478255</v>
       </c>
       <c r="F593" t="n">
-        <v>118745</v>
+        <v>115054</v>
       </c>
     </row>
     <row r="594">
@@ -14683,13 +14683,13 @@
         </is>
       </c>
       <c r="D594" t="n">
-        <v>10.35</v>
+        <v>10.225</v>
       </c>
       <c r="E594" t="n">
-        <v>91202</v>
+        <v>90098</v>
       </c>
       <c r="F594" t="n">
-        <v>8711</v>
+        <v>8606</v>
       </c>
     </row>
     <row r="595">
@@ -14707,13 +14707,13 @@
         </is>
       </c>
       <c r="D595" t="n">
-        <v>4.71</v>
+        <v>4.604</v>
       </c>
       <c r="E595" t="n">
-        <v>37455</v>
+        <v>36571</v>
       </c>
       <c r="F595" t="n">
-        <v>3961</v>
+        <v>3868</v>
       </c>
     </row>
     <row r="596">
@@ -14731,13 +14731,13 @@
         </is>
       </c>
       <c r="D596" t="n">
-        <v>18.28</v>
+        <v>17.922</v>
       </c>
       <c r="E596" t="n">
-        <v>156542</v>
+        <v>153476</v>
       </c>
       <c r="F596" t="n">
-        <v>11215</v>
+        <v>10995</v>
       </c>
     </row>
     <row r="597">
@@ -14755,13 +14755,13 @@
         </is>
       </c>
       <c r="D597" t="n">
-        <v>12.21</v>
+        <v>12.044</v>
       </c>
       <c r="E597" t="n">
-        <v>96528</v>
+        <v>95191</v>
       </c>
       <c r="F597" t="n">
-        <v>7122</v>
+        <v>7023</v>
       </c>
     </row>
     <row r="598">
@@ -14779,13 +14779,13 @@
         </is>
       </c>
       <c r="D598" t="n">
-        <v>11.97</v>
+        <v>11.473</v>
       </c>
       <c r="E598" t="n">
-        <v>939717</v>
+        <v>900422</v>
       </c>
       <c r="F598" t="n">
-        <v>78710</v>
+        <v>75419</v>
       </c>
     </row>
     <row r="599">
@@ -14803,13 +14803,13 @@
         </is>
       </c>
       <c r="D599" t="n">
-        <v>8.699999999999999</v>
+        <v>8.545</v>
       </c>
       <c r="E599" t="n">
-        <v>542694</v>
+        <v>533161</v>
       </c>
       <c r="F599" t="n">
-        <v>42030</v>
+        <v>41291</v>
       </c>
     </row>
     <row r="600">
@@ -14827,13 +14827,13 @@
         </is>
       </c>
       <c r="D600" t="n">
-        <v>4.36</v>
+        <v>4.254</v>
       </c>
       <c r="E600" t="n">
-        <v>302521</v>
+        <v>295499</v>
       </c>
       <c r="F600" t="n">
-        <v>29518</v>
+        <v>28833</v>
       </c>
     </row>
     <row r="601">
@@ -14851,13 +14851,13 @@
         </is>
       </c>
       <c r="D601" t="n">
-        <v>12.26</v>
+        <v>11.84</v>
       </c>
       <c r="E601" t="n">
-        <v>457808</v>
+        <v>442173</v>
       </c>
       <c r="F601" t="n">
-        <v>32718</v>
+        <v>31600</v>
       </c>
     </row>
   </sheetData>

</xml_diff>